<commit_message>
Use official BLS SOC 2018 titles for all 6-digit SOC files
SOC codes without an O*NET .00 code (e.g. 15-1299, Computer Occupations,
All Other) were labeled with the first 8-digit O*NET title (Web
Administrators). Titles now come from the BLS 2010-2018 crosswalk.
Values are unchanged (diffs below 1e-15). Papers 20 and 23 updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/table/25_kor_ai_usage_index.xlsx
+++ b/results/table/25_kor_ai_usage_index.xlsx
@@ -3609,7 +3609,7 @@
         <v>269116.54134640249</v>
       </c>
       <c r="P9" s="1">
-        <v>1228208.0076510101</v>
+        <v>1228208.0076510098</v>
       </c>
       <c r="Q9" s="1">
         <v>269116.54134640249</v>
@@ -3627,19 +3627,19 @@
         <v>83.973536184535234</v>
       </c>
       <c r="V9" s="1">
-        <v>232.74834247132875</v>
+        <v>232.74834247132873</v>
       </c>
       <c r="W9" s="1">
-        <v>256.06747673995483</v>
+        <v>256.06747673995477</v>
       </c>
       <c r="X9" s="1">
-        <v>232.74834247132875</v>
+        <v>232.74834247132873</v>
       </c>
       <c r="Y9" s="1">
         <v>122.04007137223037</v>
       </c>
       <c r="Z9" s="1">
-        <v>321.61015169142246</v>
+        <v>321.6101516914224</v>
       </c>
       <c r="AA9" s="1">
         <v>78.351353614503267</v>
@@ -3648,13 +3648,13 @@
         <v>89.595718754567187</v>
       </c>
       <c r="AC9" s="1">
-        <v>211.4748775503239</v>
+        <v>211.47487755032387</v>
       </c>
       <c r="AD9" s="1">
         <v>254.02180739233353</v>
       </c>
       <c r="AE9" s="1">
-        <v>273.83110711208502</v>
+        <v>273.83110711208496</v>
       </c>
       <c r="AF9" s="1">
         <v>37.894188302590699</v>
@@ -3693,7 +3693,7 @@
         <v>251098.69433398056</v>
       </c>
       <c r="AR9" s="1">
-        <v>1115948.3898637013</v>
+        <v>1115948.3898637011</v>
       </c>
       <c r="AS9" s="1">
         <v>251098.69433398056</v>
@@ -4575,7 +4575,7 @@
         <v>706487.71628364036</v>
       </c>
       <c r="P15" s="1">
-        <v>2273221.5968306167</v>
+        <v>2273221.5968306162</v>
       </c>
       <c r="Q15" s="1">
         <v>706487.71628364036</v>
@@ -4593,19 +4593,19 @@
         <v>46.872505648261019</v>
       </c>
       <c r="V15" s="1">
-        <v>79.219788014003583</v>
+        <v>79.219788014003569</v>
       </c>
       <c r="W15" s="1">
-        <v>87.156845068054167</v>
+        <v>87.156845068054139</v>
       </c>
       <c r="X15" s="1">
-        <v>79.219788014003583</v>
+        <v>79.219788014003569</v>
       </c>
       <c r="Y15" s="1">
         <v>56.185303568440396</v>
       </c>
       <c r="Z15" s="1">
-        <v>95.594454115702376</v>
+        <v>95.594454115702348</v>
       </c>
       <c r="AA15" s="1">
         <v>50.502593448018338</v>
@@ -4620,7 +4620,7 @@
         <v>76.327899284272576</v>
       </c>
       <c r="AE15" s="1">
-        <v>193.05826933171741</v>
+        <v>193.05826933171738</v>
       </c>
       <c r="AF15" s="1">
         <v>43.81339269957153</v>
@@ -4671,7 +4671,7 @@
         <v>651773.0727182863</v>
       </c>
       <c r="AV15" s="1">
-        <v>2190238.4927241844</v>
+        <v>2190238.4927241839</v>
       </c>
       <c r="AW15" s="1">
         <v>651773.0727182863</v>
@@ -4897,7 +4897,7 @@
         <v>294699.48448281607</v>
       </c>
       <c r="P17" s="1">
-        <v>1878917.0054139355</v>
+        <v>1878917.0054139353</v>
       </c>
       <c r="Q17" s="1">
         <v>294699.48448281607</v>
@@ -4915,13 +4915,13 @@
         <v>224.40214616457155</v>
       </c>
       <c r="V17" s="1">
-        <v>776.76767149601517</v>
+        <v>776.76767149601505</v>
       </c>
       <c r="W17" s="1">
-        <v>854.59228427225821</v>
+        <v>854.5922842722581</v>
       </c>
       <c r="X17" s="1">
-        <v>776.76767149601517</v>
+        <v>776.76767149601505</v>
       </c>
       <c r="Y17" s="1">
         <v>111.2594136436733</v>
@@ -4936,13 +4936,13 @@
         <v>236.45587113269855</v>
       </c>
       <c r="AC17" s="1">
-        <v>729.76726887210816</v>
+        <v>729.76726887210805</v>
       </c>
       <c r="AD17" s="1">
         <v>823.76807411992206</v>
       </c>
       <c r="AE17" s="1">
-        <v>382.54230584312313</v>
+        <v>382.54230584312307</v>
       </c>
       <c r="AF17" s="1">
         <v>42.388623773571965</v>
@@ -4981,7 +4981,7 @@
         <v>278869.74936254881</v>
       </c>
       <c r="AR17" s="1">
-        <v>1765228.1136230603</v>
+        <v>1765228.1136230601</v>
       </c>
       <c r="AS17" s="1">
         <v>278869.74936254881</v>
@@ -5154,7 +5154,7 @@
         <v>6851724.185927094</v>
       </c>
       <c r="AV18" s="1">
-        <v>42886007.865918726</v>
+        <v>42886007.865918733</v>
       </c>
       <c r="AW18" s="1">
         <v>6851724.185927094</v>
@@ -5786,7 +5786,7 @@
         <v>34480583.576332942</v>
       </c>
       <c r="AR22" s="1">
-        <v>182887067.57657853</v>
+        <v>182887067.5765785</v>
       </c>
       <c r="AS22" s="1">
         <v>34480583.576332942</v>
@@ -5863,7 +5863,7 @@
         <v>13284484.690971274</v>
       </c>
       <c r="P23" s="1">
-        <v>56028937.615912452</v>
+        <v>56028937.615912437</v>
       </c>
       <c r="Q23" s="1">
         <v>13284484.690971274</v>
@@ -5881,19 +5881,19 @@
         <v>397.80192483624455</v>
       </c>
       <c r="V23" s="1">
-        <v>934.92006647859432</v>
+        <v>934.92006647859421</v>
       </c>
       <c r="W23" s="1">
-        <v>991.07832532741145</v>
+        <v>991.07832532741133</v>
       </c>
       <c r="X23" s="1">
-        <v>934.92006647859432</v>
+        <v>934.92006647859421</v>
       </c>
       <c r="Y23" s="1">
         <v>309.1534542977667</v>
       </c>
       <c r="Z23" s="1">
-        <v>741.66605303115239</v>
+        <v>741.66605303115216</v>
       </c>
       <c r="AA23" s="1">
         <v>395.53956910069576</v>
@@ -5902,13 +5902,13 @@
         <v>400.06428057179323</v>
       </c>
       <c r="AC23" s="1">
-        <v>930.25964431990701</v>
+        <v>930.25964431990667</v>
       </c>
       <c r="AD23" s="1">
         <v>939.58048863728175</v>
       </c>
       <c r="AE23" s="1">
-        <v>253.05733230582385</v>
+        <v>253.05733230582373</v>
       </c>
       <c r="AF23" s="1">
         <v>41.299548683172205</v>
@@ -5947,7 +5947,7 @@
         <v>13208933.950117517</v>
       </c>
       <c r="AR23" s="1">
-        <v>55749642.613317817</v>
+        <v>55749642.613317803</v>
       </c>
       <c r="AS23" s="1">
         <v>13208933.950117517</v>
@@ -7109,7 +7109,7 @@
         <v>5902608.9812263707</v>
       </c>
       <c r="P31" s="1">
-        <v>25420775.090889156</v>
+        <v>25420775.090889148</v>
       </c>
       <c r="Q31" s="1">
         <v>5902608.9812263707</v>
@@ -7127,19 +7127,19 @@
         <v>48.251287749969123</v>
       </c>
       <c r="V31" s="1">
-        <v>115.83177238615778</v>
+        <v>115.83177238615777</v>
       </c>
       <c r="W31" s="1">
-        <v>122.7894909011535</v>
+        <v>122.78949090115346</v>
       </c>
       <c r="X31" s="1">
-        <v>115.787687021132</v>
+        <v>115.78768702113196</v>
       </c>
       <c r="Y31" s="1">
         <v>38.31637622086928</v>
       </c>
       <c r="Z31" s="1">
-        <v>91.144100402593878</v>
+        <v>91.14410040259385</v>
       </c>
       <c r="AA31" s="1">
         <v>48.706769394010543</v>
@@ -7148,13 +7148,13 @@
         <v>47.795806105927696</v>
       </c>
       <c r="AC31" s="1">
-        <v>115.59863177821077</v>
+        <v>115.59863177821074</v>
       </c>
       <c r="AD31" s="1">
-        <v>116.0649129941048</v>
+        <v>116.06491299410477</v>
       </c>
       <c r="AE31" s="1">
-        <v>258.40209139797241</v>
+        <v>258.4020913979723</v>
       </c>
       <c r="AF31" s="1">
         <v>41.28679895300111</v>
@@ -7193,7 +7193,7 @@
         <v>5958328.3240309441</v>
       </c>
       <c r="AR31" s="1">
-        <v>25369609.380159836</v>
+        <v>25369609.380159833</v>
       </c>
       <c r="AS31" s="1">
         <v>5958328.3240309441</v>
@@ -7205,7 +7205,7 @@
         <v>5846889.6384217972</v>
       </c>
       <c r="AV31" s="1">
-        <v>25471940.801618472</v>
+        <v>25471940.801618468</v>
       </c>
       <c r="AW31" s="1">
         <v>5846889.6384217972</v>
@@ -8355,7 +8355,7 @@
         <v>94063.715560673212</v>
       </c>
       <c r="P39" s="1">
-        <v>177224.44318477402</v>
+        <v>177224.44318477399</v>
       </c>
       <c r="Q39" s="1">
         <v>94063.715560673212</v>
@@ -8373,10 +8373,10 @@
         <v>0.31561217346070225</v>
       </c>
       <c r="V39" s="1">
-        <v>0.34571554456269649</v>
+        <v>0.34571554456269643</v>
       </c>
       <c r="W39" s="1">
-        <v>0.36648179371674244</v>
+        <v>0.36648179371674233</v>
       </c>
       <c r="X39" s="1">
         <v>0.34548846398626154</v>
@@ -8397,10 +8397,10 @@
         <v>0.33206107663384621</v>
       </c>
       <c r="AD39" s="1">
-        <v>0.35937001249154671</v>
+        <v>0.3593700124915466</v>
       </c>
       <c r="AE39" s="1">
-        <v>113.04536002756149</v>
+        <v>113.04536002756147</v>
       </c>
       <c r="AF39" s="1">
         <v>39.58417166476643</v>
@@ -8451,7 +8451,7 @@
         <v>94681.907149841703</v>
       </c>
       <c r="AV39" s="1">
-        <v>184224.14427931354</v>
+        <v>184224.14427931351</v>
       </c>
       <c r="AW39" s="1">
         <v>94681.907149841703</v>
@@ -8880,7 +8880,7 @@
         <v>4.1367340883890327</v>
       </c>
       <c r="AD42" s="1">
-        <v>4.1225898015223565</v>
+        <v>4.1225898015223557</v>
       </c>
       <c r="AE42" s="1">
         <v>118.14531276388307</v>
@@ -8934,7 +8934,7 @@
         <v>1045927.4121593426</v>
       </c>
       <c r="AV42" s="1">
-        <v>2027416.311475459</v>
+        <v>2027416.3114754588</v>
       </c>
       <c r="AW42" s="1">
         <v>1045927.4121593426</v>
@@ -10609,7 +10609,7 @@
         <v>1239235.7233420187</v>
       </c>
       <c r="P53" s="1">
-        <v>7667397.416625414</v>
+        <v>7667397.4166254122</v>
       </c>
       <c r="Q53" s="1">
         <v>1239235.7233420187</v>
@@ -10627,19 +10627,19 @@
         <v>39.513787906993691</v>
       </c>
       <c r="V53" s="1">
-        <v>137.03452293973783</v>
+        <v>137.0345229397378</v>
       </c>
       <c r="W53" s="1">
         <v>145.2658364887771</v>
       </c>
       <c r="X53" s="1">
-        <v>136.98244536249607</v>
+        <v>136.98244536249601</v>
       </c>
       <c r="Y53" s="1">
         <v>33.964334676364572</v>
       </c>
       <c r="Z53" s="1">
-        <v>120.69466535440905</v>
+        <v>120.69466535440903</v>
       </c>
       <c r="AA53" s="1">
         <v>40.243113627591569</v>
@@ -10648,13 +10648,13 @@
         <v>38.784462186395814</v>
       </c>
       <c r="AC53" s="1">
-        <v>139.56417808912985</v>
+        <v>139.5641780891298</v>
       </c>
       <c r="AD53" s="1">
-        <v>134.5048677903458</v>
+        <v>134.50486779034577</v>
       </c>
       <c r="AE53" s="1">
-        <v>371.23191038817129</v>
+        <v>371.23191038817117</v>
       </c>
       <c r="AF53" s="1">
         <v>41.058015454254004</v>
@@ -10672,7 +10672,7 @@
         <v>0.428073067086788</v>
       </c>
       <c r="AK53" s="1">
-        <v>240.68817742622778</v>
+        <v>240.68817742622772</v>
       </c>
       <c r="AL53" s="1">
         <v>36486.382999999994</v>
@@ -10693,7 +10693,7 @@
         <v>1262108.9160879129</v>
       </c>
       <c r="AR53" s="1">
-        <v>7808937.4529703502</v>
+        <v>7808937.4529703483</v>
       </c>
       <c r="AS53" s="1">
         <v>1262108.9160879129</v>
@@ -10705,7 +10705,7 @@
         <v>1216362.5305961245</v>
       </c>
       <c r="AV53" s="1">
-        <v>7525857.380280477</v>
+        <v>7525857.3802804751</v>
       </c>
       <c r="AW53" s="1">
         <v>1216362.5305961245</v>
@@ -11155,7 +11155,7 @@
         <v>0.64597069941279206</v>
       </c>
       <c r="AK56" s="1">
-        <v>383.73237521378951</v>
+        <v>383.7323752137894</v>
       </c>
       <c r="AL56" s="1">
         <v>93747.913000000088</v>
@@ -12499,7 +12499,7 @@
         <v>2290014.951667286</v>
       </c>
       <c r="P65" s="1">
-        <v>14702154.542208245</v>
+        <v>14702154.542208243</v>
       </c>
       <c r="Q65" s="1">
         <v>2290014.951667286</v>
@@ -12517,13 +12517,13 @@
         <v>234.80743779666409</v>
       </c>
       <c r="V65" s="1">
-        <v>863.44378669474474</v>
+        <v>863.44378669474452</v>
       </c>
       <c r="W65" s="1">
-        <v>915.30864810182049</v>
+        <v>915.30864810182027</v>
       </c>
       <c r="X65" s="1">
-        <v>863.44378669474474</v>
+        <v>863.44378669474452</v>
       </c>
       <c r="Y65" s="1">
         <v>203.01734569472927</v>
@@ -12538,13 +12538,13 @@
         <v>230.04796996755189</v>
       </c>
       <c r="AC65" s="1">
-        <v>885.48529202993188</v>
+        <v>885.48529202993166</v>
       </c>
       <c r="AD65" s="1">
         <v>841.40228135955761</v>
       </c>
       <c r="AE65" s="1">
-        <v>385.20677425719202</v>
+        <v>385.20677425719197</v>
       </c>
       <c r="AF65" s="1">
         <v>40.179606420188136</v>
@@ -12562,7 +12562,7 @@
         <v>0.54373990930919347</v>
       </c>
       <c r="AK65" s="1">
-        <v>292.85790705980452</v>
+        <v>292.85790705980446</v>
       </c>
       <c r="AL65" s="1">
         <v>11279.898000000003</v>
@@ -12583,7 +12583,7 @@
         <v>2336432.7849051105</v>
       </c>
       <c r="AR65" s="1">
-        <v>15077462.839950845</v>
+        <v>15077462.839950843</v>
       </c>
       <c r="AS65" s="1">
         <v>2336432.7849051105</v>
@@ -25576,7 +25576,7 @@
         <v>217090.32339002594</v>
       </c>
       <c r="P154" s="1">
-        <v>680371.29877319676</v>
+        <v>680371.29877319653</v>
       </c>
       <c r="Q154" s="1">
         <v>217090.32339002594</v>
@@ -25594,19 +25594,19 @@
         <v>1.2544430608745676</v>
       </c>
       <c r="V154" s="1">
-        <v>2.3430479382401663</v>
+        <v>2.3430479382401654</v>
       </c>
       <c r="W154" s="1">
-        <v>2.3279652820418923</v>
+        <v>2.3279652820418919</v>
       </c>
       <c r="X154" s="1">
-        <v>2.3387243671261717</v>
+        <v>2.3387243671261708</v>
       </c>
       <c r="Y154" s="1">
         <v>1.2207319884186123</v>
       </c>
       <c r="Z154" s="1">
-        <v>2.4018458548588586</v>
+        <v>2.4018458548588582</v>
       </c>
       <c r="AA154" s="1">
         <v>1.4944695908237324</v>
@@ -25615,13 +25615,13 @@
         <v>1.0144165309254027</v>
       </c>
       <c r="AC154" s="1">
-        <v>2.791369335728104</v>
+        <v>2.7913693357281035</v>
       </c>
       <c r="AD154" s="1">
-        <v>1.894726540752228</v>
+        <v>1.8947265407522278</v>
       </c>
       <c r="AE154" s="1">
-        <v>188.04282608695655</v>
+        <v>188.0428260869565</v>
       </c>
       <c r="AF154" s="1">
         <v>38.61539931528749</v>
@@ -25639,7 +25639,7 @@
         <v>0.20645625711217916</v>
       </c>
       <c r="AK154" s="1">
-        <v>71.10967391304348</v>
+        <v>71.109673913043466</v>
       </c>
       <c r="AL154" s="1">
         <v>177836.18799999982</v>
@@ -25660,7 +25660,7 @@
         <v>258628.62722704659</v>
       </c>
       <c r="AR154" s="1">
-        <v>810554.29951273056</v>
+        <v>810554.29951273045</v>
       </c>
       <c r="AS154" s="1">
         <v>258628.62722704659</v>
@@ -25672,7 +25672,7 @@
         <v>175552.01955300532</v>
       </c>
       <c r="AV154" s="1">
-        <v>550188.29803366284</v>
+        <v>550188.29803366272</v>
       </c>
       <c r="AW154" s="1">
         <v>175552.01955300532</v>
@@ -27982,7 +27982,7 @@
         <v>600.64198479468826</v>
       </c>
       <c r="T7" s="1">
-        <v>611.94121468616765</v>
+        <v>611.94121468616777</v>
       </c>
       <c r="U7" s="1">
         <v>324.53028649409003</v>
@@ -28033,7 +28033,7 @@
         <v>113038256.77727461</v>
       </c>
       <c r="AK7" s="1">
-        <v>115164723.59476672</v>
+        <v>115164723.59476674</v>
       </c>
       <c r="AL7" s="1">
         <v>21114623.27212587</v>
@@ -28202,25 +28202,25 @@
         <v>18131208.072508894</v>
       </c>
       <c r="J9" s="1">
-        <v>86776253.068478152</v>
+        <v>86776253.068478137</v>
       </c>
       <c r="K9" s="1">
         <v>18.934487990966101</v>
       </c>
       <c r="L9" s="1">
-        <v>50.846925073312995</v>
+        <v>50.846925073312988</v>
       </c>
       <c r="M9" s="1">
-        <v>53.901169903770821</v>
+        <v>53.901169903770807</v>
       </c>
       <c r="N9" s="1">
-        <v>50.776092022510255</v>
+        <v>50.776092022510241</v>
       </c>
       <c r="O9" s="1">
         <v>15.613864891343168</v>
       </c>
       <c r="P9" s="1">
-        <v>41.900810466600589</v>
+        <v>41.900810466600582</v>
       </c>
       <c r="Q9" s="1">
         <v>19.213767394615758</v>
@@ -28235,7 +28235,7 @@
         <v>50.776426696004876</v>
       </c>
       <c r="U9" s="1">
-        <v>287.16096375304755</v>
+        <v>287.1609637530475</v>
       </c>
       <c r="V9" s="1">
         <v>41.015523117354014</v>
@@ -28280,7 +28280,7 @@
         <v>17863776.865477894</v>
       </c>
       <c r="AJ9" s="1">
-        <v>86896566.834185451</v>
+        <v>86896566.834185436</v>
       </c>
       <c r="AK9" s="1">
         <v>86655939.302770853</v>
@@ -28729,7 +28729,7 @@
         <v>78.442487254103966</v>
       </c>
       <c r="S13" s="1">
-        <v>222.3136202533793</v>
+        <v>222.31362025337927</v>
       </c>
       <c r="T13" s="1">
         <v>241.08149541595498</v>
@@ -28750,7 +28750,7 @@
         <v>0.43897721606944995</v>
       </c>
       <c r="Z13" s="1">
-        <v>275.63536676577553</v>
+        <v>275.63536676577547</v>
       </c>
       <c r="AA13" t="s">
         <v>649</v>
@@ -28780,7 +28780,7 @@
         <v>5031396.2832152694</v>
       </c>
       <c r="AJ13" s="1">
-        <v>25329517.746283792</v>
+        <v>25329517.746283788</v>
       </c>
       <c r="AK13" s="1">
         <v>27467853.789071854</v>
@@ -33562,25 +33562,25 @@
         <v>222784.96468195721</v>
       </c>
       <c r="J53" s="1">
-        <v>697131.8935711931</v>
+        <v>697131.89357119286</v>
       </c>
       <c r="K53" s="1">
         <v>0.3586321647814511</v>
       </c>
       <c r="L53" s="1">
-        <v>0.61609519679751801</v>
+        <v>0.6160951967975179</v>
       </c>
       <c r="M53" s="1">
-        <v>0.61212927194935474</v>
+        <v>0.61212927194935463</v>
       </c>
       <c r="N53" s="1">
-        <v>0.61368751084231676</v>
+        <v>0.61368751084231665</v>
       </c>
       <c r="O53" s="1">
         <v>0.37149054754538302</v>
       </c>
       <c r="P53" s="1">
-        <v>0.66696745331348417</v>
+        <v>0.66696745331348395</v>
       </c>
       <c r="Q53" s="1">
         <v>0.42625065638222659</v>
@@ -33589,13 +33589,13 @@
         <v>0.29101367318067572</v>
       </c>
       <c r="S53" s="1">
-        <v>0.73235954051270447</v>
+        <v>0.73235954051270435</v>
       </c>
       <c r="T53" s="1">
-        <v>0.49983085308233155</v>
+        <v>0.49983085308233149</v>
       </c>
       <c r="U53" s="1">
-        <v>187.75016381372131</v>
+        <v>187.75016381372126</v>
       </c>
       <c r="V53" s="1">
         <v>41.919463979751391</v>
@@ -33640,10 +33640,10 @@
         <v>180779.85542939996</v>
       </c>
       <c r="AJ53" s="1">
-        <v>828688.806383188</v>
+        <v>828688.80638318788</v>
       </c>
       <c r="AK53" s="1">
-        <v>565574.98075919808</v>
+        <v>565574.98075919796</v>
       </c>
       <c r="AL53" s="1">
         <v>264790.07393451448</v>
@@ -35239,25 +35239,25 @@
         <v>3050486.8768163379</v>
       </c>
       <c r="J10" s="1">
-        <v>5356888.7754976079</v>
+        <v>5356888.775497607</v>
       </c>
       <c r="K10" s="1">
         <v>0.73982699098097904</v>
       </c>
       <c r="L10" s="1">
-        <v>0.88821932223928957</v>
+        <v>0.88821932223928945</v>
       </c>
       <c r="M10" s="1">
-        <v>0.88250168136333718</v>
+        <v>0.88250168136333706</v>
       </c>
       <c r="N10" s="1">
-        <v>0.88513138069306352</v>
+        <v>0.8851313806930633</v>
       </c>
       <c r="O10" s="1">
         <v>0.76092499666195856</v>
       </c>
       <c r="P10" s="1">
-        <v>0.98422549336203513</v>
+        <v>0.98422549336203491</v>
       </c>
       <c r="Q10" s="1">
         <v>0.78174375679948849</v>
@@ -35266,13 +35266,13 @@
         <v>0.69791022516246959</v>
       </c>
       <c r="S10" s="1">
-        <v>0.97003143936402214</v>
+        <v>0.97003143936402192</v>
       </c>
       <c r="T10" s="1">
         <v>0.80640720511455688</v>
       </c>
       <c r="U10" s="1">
-        <v>105.36459899978385</v>
+        <v>105.36459899978382</v>
       </c>
       <c r="V10" s="1">
         <v>33.661902289938432</v>
@@ -35311,7 +35311,7 @@
         <v>2877653.8420572234</v>
       </c>
       <c r="AH10" s="1">
-        <v>5850301.1579486923</v>
+        <v>5850301.1579486914</v>
       </c>
       <c r="AI10" s="1">
         <v>4863476.3930465225</v>

</xml_diff>